<commit_message>
feat(EXM): interaction v1 complete
</commit_message>
<xml_diff>
--- a/ExpandedMoongate/package/LangMod/EN/exm_localization.xlsx
+++ b/ExpandedMoongate/package/LangMod/EN/exm_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\ExpandedMoongate\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB9327DC-8AD4-4F99-8433-D86A0C20E890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31DC554A-A18B-42D8-BDC0-852B35F1A4D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="1770" windowWidth="26100" windowHeight="17625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15960" yWindow="2685" windowWidth="26100" windowHeight="17625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="107">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -156,9 +156,6 @@
   </si>
   <si>
     <t>Likes: {0}</t>
-  </si>
-  <si>
-    <t>Enter Map!</t>
   </si>
   <si>
     <t>View Details</t>
@@ -172,13 +169,197 @@
 {1}</t>
   </si>
   <si>
-    <t>Did you like the map?</t>
-  </si>
-  <si>
     <t>exm_ui_rate_map_dialog_yes</t>
   </si>
   <si>
     <t>I like it!</t>
+  </si>
+  <si>
+    <t>Did you like the map?
+{0}</t>
+  </si>
+  <si>
+    <t>exm_ui_last_visit</t>
+  </si>
+  <si>
+    <t>exm_ui_last_liked</t>
+  </si>
+  <si>
+    <t>you visited on {0}</t>
+  </si>
+  <si>
+    <t>you liked the map</t>
+  </si>
+  <si>
+    <t>exm_ui_sort_type</t>
+  </si>
+  <si>
+    <t>exm_ui_no_history</t>
+  </si>
+  <si>
+    <t>You haven't visited any maps this session yet</t>
+  </si>
+  <si>
+    <t>Sort By</t>
+  </si>
+  <si>
+    <t>Visit Map!</t>
+  </si>
+  <si>
+    <t>exm_ui_lang_filter</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>exm_ui_adult_filter</t>
+  </si>
+  <si>
+    <t>No Adult</t>
+  </si>
+  <si>
+    <t>最新のサーバー情報の取得に失敗しました。</t>
+  </si>
+  <si>
+    <t>合計マップ数：{0}</t>
+  </si>
+  <si>
+    <t>合計訪問数：{0}</t>
+  </si>
+  <si>
+    <t>過去24時間の新規マップ数：{0}</t>
+  </si>
+  <si>
+    <t>過去24時間の訪問数：{0}</t>
+  </si>
+  <si>
+    <t>サーバーがタイムアウトしました。</t>
+  </si>
+  <si>
+    <t>ゾーン「{0}」の作成に失敗しました</t>
+  </si>
+  <si>
+    <t>マップのメタデータの取得に失敗しました</t>
+  </si>
+  <si>
+    <t>マップ評価の更新に失敗しました</t>
+  </si>
+  <si>
+    <t>マップブラウザ</t>
+  </si>
+  <si>
+    <t>マップ履歴</t>
+  </si>
+  <si>
+    <t>訪問数：{0}</t>
+  </si>
+  <si>
+    <t>いいね：{0}</t>
+  </si>
+  <si>
+    <t>マップに行く！</t>
+  </si>
+  <si>
+    <t>詳細を見る</t>
+  </si>
+  <si>
+    <t>「Expanded Moongate」設定が変更されました</t>
+  </si>
+  <si>
+    <t>いいね！</t>
+  </si>
+  <si>
+    <t>このマップは気に入りましたか？
+{0}</t>
+  </si>
+  <si>
+    <t>{0}
+作成者：
+{1}</t>
+  </si>
+  <si>
+    <t>{0} に訪問しました</t>
+  </si>
+  <si>
+    <t>このマップにいいねしました</t>
+  </si>
+  <si>
+    <t>このセッションではまだマップを訪問していません</t>
+  </si>
+  <si>
+    <t>並び替え</t>
+  </si>
+  <si>
+    <t>成人向けなし</t>
+  </si>
+  <si>
+    <t>言語</t>
+  </si>
+  <si>
+    <t>exm_ui_sort_type_Created</t>
+  </si>
+  <si>
+    <t>最終更新</t>
+  </si>
+  <si>
+    <t>Last Updated</t>
+  </si>
+  <si>
+    <t>exm_ui_sort_type_Visits</t>
+  </si>
+  <si>
+    <t>人気順（訪問）</t>
+  </si>
+  <si>
+    <t>Most Visited</t>
+  </si>
+  <si>
+    <t>exm_ui_sort_type_Rating</t>
+  </si>
+  <si>
+    <t>人気順（いいね）</t>
+  </si>
+  <si>
+    <t>Most Liked</t>
+  </si>
+  <si>
+    <t>exm_ui_lang_filter_All</t>
+  </si>
+  <si>
+    <t>すべて</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>exm_ui_lang_filter_EN</t>
+  </si>
+  <si>
+    <t>英語</t>
+  </si>
+  <si>
+    <t>EN</t>
+  </si>
+  <si>
+    <t>exm_ui_lang_filter_CN</t>
+  </si>
+  <si>
+    <t>中国語</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>exm_ui_lang_filter_JP</t>
+  </si>
+  <si>
+    <t>日本語</t>
+  </si>
+  <si>
+    <t>JP</t>
+  </si>
+  <si>
+    <t>ムーンゲート</t>
   </si>
 </sst>
 </file>
@@ -586,7 +767,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>27</v>
@@ -597,7 +778,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>28</v>
@@ -608,7 +789,7 @@
         <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>29</v>
@@ -619,7 +800,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>30</v>
@@ -630,7 +811,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>31</v>
@@ -641,7 +822,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>32</v>
@@ -652,7 +833,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>33</v>
@@ -663,7 +844,7 @@
         <v>12</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>34</v>
@@ -674,7 +855,7 @@
         <v>13</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>35</v>
@@ -685,7 +866,7 @@
         <v>14</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>36</v>
+        <v>69</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>36</v>
@@ -697,7 +878,7 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4" t="s">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>37</v>
@@ -708,7 +889,7 @@
         <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>38</v>
@@ -719,7 +900,7 @@
         <v>17</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>39</v>
@@ -730,7 +911,7 @@
         <v>18</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>40</v>
@@ -741,10 +922,10 @@
         <v>19</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -752,10 +933,10 @@
         <v>20</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -774,7 +955,7 @@
         <v>22</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>25</v>
@@ -782,35 +963,178 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="46.5">
       <c r="A23" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="69.75">
       <c r="A24" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>44</v>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:4" s="3" customFormat="1">

</xml_diff>

<commit_message>
feat(EXM): add more filters and query ui
</commit_message>
<xml_diff>
--- a/ExpandedMoongate/package/LangMod/EN/exm_localization.xlsx
+++ b/ExpandedMoongate/package/LangMod/EN/exm_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\ExpandedMoongate\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31DC554A-A18B-42D8-BDC0-852B35F1A4D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45020CD2-6E83-4E6F-BD9A-91A33B5B9E33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15960" yWindow="2685" windowWidth="26100" windowHeight="17625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5910" yWindow="2160" windowWidth="25545" windowHeight="17625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="158">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -360,6 +360,159 @@
   </si>
   <si>
     <t>ムーンゲート</t>
+  </si>
+  <si>
+    <t>exm_ui_search_hint</t>
+  </si>
+  <si>
+    <t>Name, Author, or Map ID</t>
+  </si>
+  <si>
+    <t>exm_ui_btn_search</t>
+  </si>
+  <si>
+    <t>Search</t>
+  </si>
+  <si>
+    <t>exm_ui_btn_search_clear</t>
+  </si>
+  <si>
+    <t>Clear Result</t>
+  </si>
+  <si>
+    <t>exm_ui_map_view</t>
+  </si>
+  <si>
+    <t>exm_ui_no_map_data</t>
+  </si>
+  <si>
+    <t>Empty Map Data</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period</t>
+  </si>
+  <si>
+    <t>Time Period</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period_AllTime</t>
+  </si>
+  <si>
+    <t>All Time</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period_Today</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period_OneWeek</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period_ThirtyDays</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period_ThreeMonths</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period_OneYear</t>
+  </si>
+  <si>
+    <t>Today</t>
+  </si>
+  <si>
+    <t>One Week</t>
+  </si>
+  <si>
+    <t>30 Days</t>
+  </si>
+  <si>
+    <t>3 Months</t>
+  </si>
+  <si>
+    <t>1 year</t>
+  </si>
+  <si>
+    <t>exm_ui_time_period_SixMonths</t>
+  </si>
+  <si>
+    <t>6 Months</t>
+  </si>
+  <si>
+    <t>名前、作者、またはマップID</t>
+  </si>
+  <si>
+    <t>検索</t>
+  </si>
+  <si>
+    <t>結果をクリア</t>
+  </si>
+  <si>
+    <t>マップデータがありません</t>
+  </si>
+  <si>
+    <t>期間</t>
+  </si>
+  <si>
+    <t>全期間</t>
+  </si>
+  <si>
+    <t>今日</t>
+  </si>
+  <si>
+    <t>1週間</t>
+  </si>
+  <si>
+    <t>30日間</t>
+  </si>
+  <si>
+    <t>3ヶ月間</t>
+  </si>
+  <si>
+    <t>6ヶ月間</t>
+  </si>
+  <si>
+    <t>1年間</t>
+  </si>
+  <si>
+    <t>exm_ui_copy_name</t>
+  </si>
+  <si>
+    <t>exm_ui_copy_author</t>
+  </si>
+  <si>
+    <t>exm_ui_copy_view</t>
+  </si>
+  <si>
+    <t>Copy Author</t>
+  </si>
+  <si>
+    <t>Copy Name</t>
+  </si>
+  <si>
+    <t>Copy ID</t>
+  </si>
+  <si>
+    <t>コピーID</t>
+  </si>
+  <si>
+    <t>コピー名前</t>
+  </si>
+  <si>
+    <t>コピー作者</t>
+  </si>
+  <si>
+    <t>exm_ui_file_size</t>
+  </si>
+  <si>
+    <t>File Size : {0}</t>
+  </si>
+  <si>
+    <t>ファイルサイズ : {0}</t>
+  </si>
+  <si>
+    <t>Map ID : {0}</t>
+  </si>
+  <si>
+    <t>マップID : {0}</t>
   </si>
 </sst>
 </file>
@@ -722,7 +875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFC124"/>
+  <dimension ref="A1:XFC125"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="63.28515625" style="4" customWidth="1"/>
@@ -1137,17 +1290,193 @@
         <v>105</v>
       </c>
     </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
     <row r="39" spans="1:4" s="3" customFormat="1">
-      <c r="A39" s="4"/>
+      <c r="A39" s="4" t="s">
+        <v>109</v>
+      </c>
       <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-    </row>
-    <row r="61" spans="1:4" s="2" customFormat="1">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
+      <c r="C39" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="62" spans="1:4" s="2" customFormat="1">
       <c r="A62" s="4"/>
@@ -1155,11 +1484,17 @@
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
     </row>
-    <row r="119" spans="3:4">
-      <c r="C119" s="5"/>
-    </row>
-    <row r="124" spans="3:4">
-      <c r="D124" s="6"/>
+    <row r="63" spans="1:4" s="2" customFormat="1">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+    </row>
+    <row r="120" spans="3:4">
+      <c r="C120" s="5"/>
+    </row>
+    <row r="125" spans="3:4">
+      <c r="D125" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
fix(EXM): ui improvements & loc formatting
</commit_message>
<xml_diff>
--- a/ExpandedMoongate/package/LangMod/EN/exm_localization.xlsx
+++ b/ExpandedMoongate/package/LangMod/EN/exm_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\ExpandedMoongate\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8903B4A7-749D-4967-A1FE-F24F97458EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFCB79C-DF5B-4F79-889D-9310CD1AF276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5910" yWindow="2160" windowWidth="25545" windowHeight="17625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16665" yWindow="3270" windowWidth="25545" windowHeight="17610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -119,18 +119,6 @@
     <t>Failed to get latest server info.</t>
   </si>
   <si>
-    <t>{0} total maps</t>
-  </si>
-  <si>
-    <t>{0} total visits</t>
-  </si>
-  <si>
-    <t>{0} maps added past 24 hours</t>
-  </si>
-  <si>
-    <t>{0} visits past 24 hours</t>
-  </si>
-  <si>
     <t>Server timed out.</t>
   </si>
   <si>
@@ -150,12 +138,6 @@
   </si>
   <si>
     <t>Moongate Server</t>
-  </si>
-  <si>
-    <t>Visits: {0}</t>
-  </si>
-  <si>
-    <t>Likes: {0}</t>
   </si>
   <si>
     <t>View Details</t>
@@ -221,18 +203,6 @@
     <t>最新のサーバー情報の取得に失敗しました。</t>
   </si>
   <si>
-    <t>合計マップ数：{0}</t>
-  </si>
-  <si>
-    <t>合計訪問数：{0}</t>
-  </si>
-  <si>
-    <t>過去24時間の新規マップ数：{0}</t>
-  </si>
-  <si>
-    <t>過去24時間の訪問数：{0}</t>
-  </si>
-  <si>
     <t>サーバーがタイムアウトしました。</t>
   </si>
   <si>
@@ -249,12 +219,6 @@
   </si>
   <si>
     <t>マップ履歴</t>
-  </si>
-  <si>
-    <t>訪問数：{0}</t>
-  </si>
-  <si>
-    <t>いいね：{0}</t>
   </si>
   <si>
     <t>マップに行く！</t>
@@ -548,6 +512,42 @@
   </si>
   <si>
     <t>このまま続ける</t>
+  </si>
+  <si>
+    <t>Likes: {0:N0}</t>
+  </si>
+  <si>
+    <t>Visits: {0:N0}</t>
+  </si>
+  <si>
+    <t>訪問数：{0:N0}</t>
+  </si>
+  <si>
+    <t>いいね：{0:N0}</t>
+  </si>
+  <si>
+    <t>{0:N0} total maps</t>
+  </si>
+  <si>
+    <t>{0:N0} total visits</t>
+  </si>
+  <si>
+    <t>{0:N0} maps added past 24 hours</t>
+  </si>
+  <si>
+    <t>{0:N0} visits past 24 hours</t>
+  </si>
+  <si>
+    <t>過去24時間の訪問数：{0:N0}</t>
+  </si>
+  <si>
+    <t>過去24時間の新規マップ数：{0:N0}</t>
+  </si>
+  <si>
+    <t>合計訪問数：{0:N0}</t>
+  </si>
+  <si>
+    <t>合計マップ数：{0:N0}</t>
   </si>
 </sst>
 </file>
@@ -955,7 +955,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>27</v>
@@ -966,10 +966,10 @@
         <v>6</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>61</v>
+        <v>168</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>28</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -977,10 +977,10 @@
         <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>62</v>
+        <v>167</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>29</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -988,10 +988,10 @@
         <v>8</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>63</v>
+        <v>166</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>30</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -999,10 +999,10 @@
         <v>9</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>64</v>
+        <v>165</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>31</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1010,10 +1010,10 @@
         <v>10</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1021,10 +1021,10 @@
         <v>11</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1032,10 +1032,10 @@
         <v>12</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1043,10 +1043,10 @@
         <v>13</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1054,10 +1054,10 @@
         <v>14</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:4" s="3" customFormat="1">
@@ -1066,10 +1066,10 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1077,10 +1077,10 @@
         <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1088,10 +1088,10 @@
         <v>17</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>71</v>
+        <v>159</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>39</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1099,10 +1099,10 @@
         <v>18</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>40</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1110,10 +1110,10 @@
         <v>19</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1121,10 +1121,10 @@
         <v>20</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -1143,7 +1143,7 @@
         <v>22</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>25</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="46.5">
@@ -1165,396 +1165,396 @@
         <v>26</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="69.75">
       <c r="A24" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="4" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="4" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="4" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:4" s="3" customFormat="1">
       <c r="A39" s="4" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="4" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="4" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="4" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C49" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="D49" s="4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="4" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="4" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="4" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="4" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="4" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="4" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="46.5">
       <c r="A56" s="4" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="4" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="4" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
     </row>
     <row r="62" spans="1:4" s="2" customFormat="1">

</xml_diff>